<commit_message>
[FIX] Einvoice with SP
</commit_message>
<xml_diff>
--- a/l10n_it_einvoice_out/tests/data/account_tax.xlsx
+++ b/l10n_it_einvoice_out/tests/data/account_tax.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="105">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -298,6 +298,9 @@
     <t xml:space="preserve">Acq.fuori campo IVA (art.1 DPR633)</t>
   </si>
   <si>
+    <t xml:space="preserve">l10n_it_ade.n1</t>
+  </si>
+  <si>
     <t xml:space="preserve">z0bug.tax_a1v</t>
   </si>
   <si>
@@ -305,6 +308,9 @@
   </si>
   <si>
     <t xml:space="preserve">Vend.fuori campo IVA (art.1 DPR633)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuori campo IVA (art.1 DPR633)</t>
   </si>
   <si>
     <t xml:space="preserve">z0bug.tax_a17c2a</t>
@@ -1035,7 +1041,7 @@
       <c r="K13" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="M13" s="0" t="s">
+      <c r="M13" s="1" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1280,16 +1286,19 @@
       <c r="H22" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="K22" s="1" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D23" s="1" t="n">
         <v>60</v>
@@ -1306,16 +1315,22 @@
       <c r="H23" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="K23" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D24" s="1" t="n">
         <v>80</v>
@@ -1347,13 +1362,13 @@
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D25" s="1" t="n">
         <v>80</v>
@@ -1382,13 +1397,13 @@
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D26" s="1" t="n">
         <v>81</v>

</xml_diff>